<commit_message>
data update huawei honor
</commit_message>
<xml_diff>
--- a/data/apple-service-prices.xlsx
+++ b/data/apple-service-prices.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamd\Github\maro_web\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stano\Documents\mobilflex\dzuris.github.io\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163D0DBB-F188-4A4C-9738-6E5AEC16787E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0A221D8-CE22-4320-9652-946113E1BC52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{E889351A-8D47-49F3-90BB-9B5B0FF2FD64}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{E889351A-8D47-49F3-90BB-9B5B0FF2FD64}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -149,7 +149,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normálna" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -165,9 +165,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motív Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -205,7 +205,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -311,7 +311,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -462,28 +462,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1D3CA37-09CC-4DEA-ADDE-A1FEC67AF807}">
   <dimension ref="A1:T3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" customWidth="1"/>
+    <col min="9" max="9" width="11.109375" customWidth="1"/>
+    <col min="10" max="10" width="11.33203125" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" customWidth="1"/>
+    <col min="13" max="13" width="10.44140625" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="6.140625" customWidth="1"/>
-    <col min="16" max="16" width="11.5703125" customWidth="1"/>
-    <col min="17" max="17" width="11.7109375" customWidth="1"/>
-    <col min="19" max="19" width="12.5703125" customWidth="1"/>
+    <col min="15" max="15" width="6.109375" customWidth="1"/>
+    <col min="16" max="16" width="11.5546875" customWidth="1"/>
+    <col min="17" max="17" width="11.6640625" customWidth="1"/>
+    <col min="19" max="19" width="12.5546875" customWidth="1"/>
     <col min="20" max="20" width="13" customWidth="1"/>
-    <col min="21" max="21" width="12.28515625" customWidth="1"/>
+    <col min="21" max="21" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -545,7 +545,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -604,7 +604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>

</xml_diff>